<commit_message>
Citation Fit Check: fix the Ready wording and the page's percent rounding
Two defects from the review of PR #58.

The Ready message said "Every critical check passes", but the brief's rule
blocks Ready only on a critical No, so four critical Partials and eight
Yes reach Ready at 20. The wording now says exactly the rule: no critical
check is answered No, and the total is 20 or more. The rule is unchanged.

The page rounded ratios to whole percent with its own helper while the
workbook shows one decimal place (40% against 40.0%). It now uses the
shared percent() helper.

A unit test and a workbook variant cover the critical-Partial case;
verify_xlsx.py passes 50 of 50.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/citation-fit-check.xlsx
+++ b/downloads/citation-fit-check.xlsx
@@ -1702,7 +1702,7 @@
         <v/>
       </c>
       <c r="D5" s="7">
-        <f>IF(C5="Hold","Don’t trust these answers yet.",IF(C5="Fix first","No critical check fails, but the total is under 20. Fix the gaps before you rely on these answers.",IF(C5="Ready","Every critical check passes and the total is 20 or more.",IF(COUNTA(E11:E26)=0,"","Answer all 12 checks to see the decision."))))</f>
+        <f>IF(C5="Hold","Don’t trust these answers yet.",IF(C5="Fix first","No critical check fails, but the total is under 20. Fix the gaps before you rely on these answers.",IF(C5="Ready","No critical check is answered No, and the total is 20 or more.",IF(COUNTA(E11:E26)=0,"","Answer all 12 checks to see the decision."))))</f>
         <v/>
       </c>
     </row>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="D54" s="7">
-        <f>IF(C54="Hold","Don’t trust these answers yet.",IF(C54="Fix first","No critical check fails, but the total is under 20. Fix the gaps before you rely on these answers.",IF(C54="Ready","Every critical check passes and the total is 20 or more.",IF(COUNTA(E60:E75)=0,"","Answer all 12 checks to see the decision."))))</f>
+        <f>IF(C54="Hold","Don’t trust these answers yet.",IF(C54="Fix first","No critical check fails, but the total is under 20. Fix the gaps before you rely on these answers.",IF(C54="Ready","No critical check is answered No, and the total is 20 or more.",IF(COUNTA(E60:E75)=0,"","Answer all 12 checks to see the decision."))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Enforce the dropdowns in the three earlier tool workbooks
The Gate Routing Map, Citation Fit Check and Rework Cost Check builders
wrote every data validation with openpyxl's default showErrorMessage off,
so Excel accepted any typed value in a dropdown cell, and the Gate Routing
Map's "not this route" rule refused nothing. Each builder now switches it
on for every validation just before saving, so a rule added later is
covered too. Found in the PR #69 review.

All three workbooks rebuilt; refs.json unchanged. verify_xlsx.py 87/87,
50/50 and 40/40. 60 of 60 validations across the four tool workbooks now
refuse a wrong value. npm test 224 of 224.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/citation-fit-check.xlsx
+++ b/downloads/citation-fit-check.xlsx
@@ -1341,13 +1341,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$1:$Z$6</formula1>
     </dataValidation>
-    <dataValidation sqref="F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$8:$Z$11</formula1>
     </dataValidation>
-    <dataValidation sqref="H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$13:$Z$15</formula1>
     </dataValidation>
   </dataValidations>
@@ -1623,7 +1623,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$1:$Z$2</formula1>
     </dataValidation>
   </dataValidations>
@@ -2223,7 +2223,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E12 E13 E14 E16 E17 E18 E20 E21 E22 E23 E25 E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="E12 E13 E14 E16 E17 E18 E20 E21 E22 E23 E25 E26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$1:$Z$3</formula1>
     </dataValidation>
   </dataValidations>
@@ -2644,7 +2644,7 @@
     <mergeCell ref="A5:B5"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$1:$Z$4</formula1>
     </dataValidation>
   </dataValidations>
@@ -4522,22 +4522,22 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
-    <dataValidation sqref="E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$1:$Z$6</formula1>
     </dataValidation>
-    <dataValidation sqref="F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$8:$Z$11</formula1>
     </dataValidation>
-    <dataValidation sqref="H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$13:$Z$15</formula1>
     </dataValidation>
-    <dataValidation sqref="D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 F38 F39 F40 F41 F42 F43 F44 F45 F46 F47 G38 G39 G40 G41 G42 G43 G44 G45 G46 G47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 F38 F39 F40 F41 F42 F43 F44 F45 F46 F47 G38 G39 G40 G41 G42 G43 G44 G45 G46 G47" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$17:$Z$18</formula1>
     </dataValidation>
-    <dataValidation sqref="G87 G88 G89 G90 G91 G92 G93 G94 G95 G96 G97 G98 G99 G100 G101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="G87 G88 G89 G90 G91 G92 G93 G94 G95 G96 G97 G98 G99 G100 G101" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$20:$Z$23</formula1>
     </dataValidation>
-    <dataValidation sqref="E61 E62 E63 E65 E66 E67 E69 E70 E71 E72 E74 E75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
+    <dataValidation sqref="E61 E62 E63 E65 E66 E67 E69 E70 E71 E72 E74 E75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an option" error="Pick one of the options in the list." type="list">
       <formula1>$Z$25:$Z$27</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>